<commit_message>
Dopisz sprawdzenie 30 miast sredniej wielkosci (odpowiedz na pytanie o luke geograficzna) - 10 nowych firm, 15 z 30 miast bez trafienia, wniosek: dalsze rozszerzanie ma malejace zwroty. Zaktualizowano plik md i Excel
</commit_message>
<xml_diff>
--- a/plany/lista-konkurencji-KRS-Guard-2026-08-05.xlsx
+++ b/plany/lista-konkurencji-KRS-Guard-2026-08-05.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +65,11 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001A3A5C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -112,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -136,6 +141,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -501,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -562,7 +568,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -607,7 +613,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="C9" s="5" t="inlineStr"/>
     </row>
@@ -653,12 +659,20 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Dodatkowe sprawdzenie (na pytanie właściciela): 30 miast średniej wielkości poza pierwotną piętnastką największych miast dodało tylko 10 nowych firm; dla 15 z 30 miast nie znaleziono żadnej pasującej kancelarii — dalsze rozszerzanie geograficzne miałoby już malejące zwroty.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A15:F15"/>
@@ -1663,7 +1677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B80"/>
+  <dimension ref="A1:B90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2610,6 +2624,126 @@
       <c r="B80" s="4" t="inlineStr">
         <is>
           <t>Warszawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>Kancelaria Adwokacka Tomasz Diduch</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Gliwice</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>Kancelaria Adwokacka Gatner &amp; Gatner</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>Bielsko-Biała</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>Kancelaria STERRN - oddział Zabrze</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Zabrze</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>Kancelaria STERRN - oddział Ruda Śląska</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>Ruda Śląska</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>Adwokat Mikołaj Jarosiński</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Tychy (+ Katowice/Gliwice/Żory/Rybnik)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>Adwokat Seweryn Pytlewski</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Dąbrowa Górnicza</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>Kancelaria Radcy Prawnego (KRP Wałbrzych)</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Wałbrzych</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>Kancelaria Adwokacka Andrzej Turczyn</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>Koszalin</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t>Kancelaria ILT</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>Legnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
+        <is>
+          <t>Kancelaria Radcy Prawnego Łukasz Pryzwan (niepewne, raczej strona wierzyciela)</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>Słupsk</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Zweryfikuj konkurencje Tier 1 z pierwszej reki + dodaj analize SWOT
</commit_message>
<xml_diff>
--- a/plany/lista-konkurencji-KRS-Guard-2026-08-05.xlsx
+++ b/plany/lista-konkurencji-KRS-Guard-2026-08-05.xlsx
@@ -117,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -142,6 +142,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -663,6 +669,13 @@
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Dodatkowe sprawdzenie (na pytanie właściciela): 30 miast średniej wielkości poza pierwotną piętnastką największych miast dodało tylko 10 nowych firm; dla 15 z 30 miast nie znaleziono żadnej pasującej kancelarii — dalsze rozszerzanie geograficzne miałoby już malejące zwroty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Aktualizacja 05.08.2026: opisy Tier 1 zweryfikowane z pierwszej reki (odwiedzenie realnych stron WWW, nie tylko domysl) + dodane opinie klientow, status radcy prawnego i pelna analiza SWOT (mocne/slabe strony konkurenta, szanse/zagrozenia dla KRS Guard) dla kazdej z 21 firm Tier 1.</t>
         </is>
       </c>
     </row>
@@ -687,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -698,6 +711,14 @@
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="12" max="12"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
+    <col width="46" customWidth="1" min="14" max="14"/>
+    <col width="46" customWidth="1" min="15" max="15"/>
+    <col width="46" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -741,8 +762,48 @@
           <t>Liczba spraw / klientów (ogólne, nie tylko ten temat)</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="60" customHeight="1">
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>Firmowana przez radce prawnego / tytul zawodowy</t>
+        </is>
+      </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
+          <t>Opinie klientow</t>
+        </is>
+      </c>
+      <c r="K1" s="12" t="inlineStr">
+        <is>
+          <t>Ciekawe pomysly dla KRS Guard</t>
+        </is>
+      </c>
+      <c r="L1" s="12" t="inlineStr">
+        <is>
+          <t>Ocena wiarygodnosci opisu (weryfikacja 05.08.2026)</t>
+        </is>
+      </c>
+      <c r="M1" s="12" t="inlineStr">
+        <is>
+          <t>SWOT: Mocne strony konkurenta</t>
+        </is>
+      </c>
+      <c r="N1" s="12" t="inlineStr">
+        <is>
+          <t>SWOT: Słabe strony konkurenta</t>
+        </is>
+      </c>
+      <c r="O1" s="12" t="inlineStr">
+        <is>
+          <t>SWOT: Szanse dla KRS Guard</t>
+        </is>
+      </c>
+      <c r="P1" s="12" t="inlineStr">
+        <is>
+          <t>SWOT: Zagrożenia dla KRS Guard</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="150" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Kancelaria Prawna Skarbiec (Robert Nogacki)</t>
@@ -760,7 +821,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Art. 299 KSH + postępowania przed US i ZUS + bezpieczne wyjście z zarządu — najszerszy zakres tematyczny ze wszystkich znalezionych</t>
+          <t>Szersza tresc niz wskazywalby jednorazowy przeglad strony: dedykowana podstrona "Ochrona prawna czlonkow zarzadu" (kancelaria-skarbiec.pl/odpowiedzialnosc-czlonka-zarzadu/) z sekcja o bezpiecznym wyjsciu z zarzadu i wzmianka o art. 116 Ordynacji (US), plus osobny dedykowany artykul o art. 299 KSH (kancelaria-skarbiec.pl/odpowiedzialnosc-czlonkow-zarzadu-sp-z-o-o/) z pelna systematyka linii obrony i cytatem wyroku TK P 5/19.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -783,8 +844,48 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="60" customHeight="1">
+      <c r="I2" s="13" t="inlineStr">
+        <is>
+          <t>TAK - Robert Nogacki, radca prawny, OIRP Warszawa nr WA-9026.</t>
+        </is>
+      </c>
+      <c r="J2" s="13" t="inlineStr">
+        <is>
+          <t>Osobna podstrona /opinie-klientow/, ale to tekst pisany z perspektywy kancelarii (brak imiennych cytatow/zrzutow ekranu) + samodeklarowana ocena 5.0/5.0 na Facebooku.</t>
+        </is>
+      </c>
+      <c r="K2" s="13" t="inlineStr">
+        <is>
+          <t>Podstrona "Opinie klientow" wprost i transparentnie odpowiada na krytyke (cena, zarzuty o falszywe opinie) zamiast ja ukrywac - buduje wiarygodnosc inaczej niz zwykle gwiazdki.</t>
+        </is>
+      </c>
+      <c r="L2" s="13" t="inlineStr">
+        <is>
+          <t>ROZBIEZNOSC Z OBSERWACJA WLASCICIELA: przy weryfikacji 05.08 tresc okazala sie SZERSZA, nie wezsza, niz zglosil wlasciciel po wlasnej wizycie na stronie. Mozliwe, ze trafil na inna podstrone / strone glowna. Rekomendacja: sprawdzic ponownie oba wskazane adresy URL.</t>
+        </is>
+      </c>
+      <c r="M2" s="13" t="inlineStr">
+        <is>
+          <t>Bardzo szeroka, dogłębna treść merytoryczna (2 dedykowane artykuły), rozpoznawalna marka (Robert Nogacki, ~20 lat na rynku), transparentna podstrona "Opinie klientów" wprost adresująca krytykę zamiast jej ukrywać.</t>
+        </is>
+      </c>
+      <c r="N2" s="13" t="inlineStr">
+        <is>
+          <t>Brak cen na stronie, niejasny sposób pierwszego kontaktu, wyłącznie/głównie stacjonarnie (Warszawa) — brak modelu zdalnego, brak liczby spraw specyficznej dla ochrony zarządu, opinie klientów bez imiennych cytatów.</t>
+        </is>
+      </c>
+      <c r="O2" s="13" t="inlineStr">
+        <is>
+          <t>Brak jawnego cennika i pracy zdalnej — KRS Guard może wprost kontrastować "jasna cena od pierwszego kontaktu" i "zdalnie w całej Polsce, bez biura".</t>
+        </is>
+      </c>
+      <c r="P2" s="13" t="inlineStr">
+        <is>
+          <t>Silna, rozpoznawalna marka i wysoka pozycja SEO/zaufania mogą dominować wyniki wyszukiwania mimo braku transparentności cenowej.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="150" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Kancelaria MW (Maciej Wieczorkowski)</t>
@@ -802,7 +903,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Art. 299 KSH + wzmianka o US/ZUS + rezygnacja z funkcji</t>
+          <t>Jeden obszerny wpis blogowy o art. 299 KSH (kancelariamw.pl/art-299-ksh-odpowiedzialnosc-czlonkow-zarzadu-sp-z-o-o/), zapowiedziany jako pierwszy z cyklu "kompendium wiedzy". Art. 299 KSH NIE figuruje wsrod glownych specjalizacji na stronie glownej (IT, cywilne, spadkowe, obsluga firm, upadlosci, IP, rodzinne, karne). Brak znalezionych wzmianek o US/ZUS lub o "bezpiecznym odejsciu z zarzadu" jako osobnym temacie.</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -825,8 +926,48 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="60" customHeight="1">
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>NIE - adwokat (Pomorska Izba Adwokacka w Gdansku), nie radca prawny.</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>Brak na stronie - odeslanie do opinii na Google My Business.</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>Format "kompendium wiedzy" jako zapowiedziany cykl edukacyjny o prawie spolek (choc w tym przypadku wyglada na porzucony po jednym wpisie).</t>
+        </is>
+      </c>
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>CZESCIOWO ZAWYZONE: art. 299 potwierdzony, ale watek US/ZUS i rezygnacji z funkcji - nie znaleziony na stronie.</t>
+        </is>
+      </c>
+      <c r="M3" s="13" t="inlineStr">
+        <is>
+          <t>Solidny merytorycznie artykuł o art. 299 KSH, lokalna obecność na rynku trójmiejskim/kujawskim.</t>
+        </is>
+      </c>
+      <c r="N3" s="13" t="inlineStr">
+        <is>
+          <t>Temat to pojedynczy, porzucony wpis blogowy — nie stała oferta; brak wątku ZUS/US i "bezpiecznego odejścia z zarządu"; adwokat, nie radca prawny; brak cen; brak opinii na stronie.</t>
+        </is>
+      </c>
+      <c r="O3" s="13" t="inlineStr">
+        <is>
+          <t>Wąski, niepełny zakres tematyczny (brak US/ZUS) — KRS Guard może pozycjonować się jako kompleksowe rozwiązanie (3 zagrożenia w 1 produkcie) wobec klientów szukających szerzej.</t>
+        </is>
+      </c>
+      <c r="P3" s="13" t="inlineStr">
+        <is>
+          <t>Niskie — mały, lokalny zasięg, temat wygląda na poboczny wątek działalności.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="150" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Bladowski.Legal</t>
@@ -844,7 +985,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Cała sekcja serwisu: art. 299/586 KSH, doradztwo kryzysowe, ochrona majątku prywatnego, darmowy poradnik PDF jako lead magnet</t>
+          <t>Cala strona zbudowana wokol art. 299/586 KSH: dedykowana sekcja "Ochrona Zarzadu przed art. 299 K.s.h.", produkty w sklepie ("Ochrona Zarzadu 299/586 K.s.h.", "Zarzad Powierniczy"), dziesiatki wpisow blogowych o 299/586 KSH, ZUS, US, komornikach. Cytat z poradnika: "Art. 299 Kodeksu spolek handlowych [...] stanowi potencjalna «bron atomowa» [...] Odpowiedzialnosc jest osobista, nielimitowana i moze dotyczyc nawet bylych czlonkow zarzadu."</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -867,8 +1008,48 @@
           <t>400+ (ogólny dorobek kancelarii)</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="60" customHeight="1">
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>NIE - Blazej Bladowski przedstawia sie jako "ekspert prawa gospodarczego", BEZ zadnego tytulu zawodowego (nie radca prawny, nie adwokat). Firma to sp.j., nie kancelaria radcowska.</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>Link "Opinie Zadowolonych Klientow" istnieje na liscie "Sukcesy", ale tresc nie zostala zweryfikowana (podstrona nie zdazyla zostac otwarta) - niepotwierdzone.</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>UWAGA ETYCZNA: glowny model biznesowy to "skup zadluzonych spolek" (im wieksze zadluzenie tym lepiej) - blisko granicy legalnosci, kojarzone ze "slupami"; ODRADZAMY inspiracje tym modelem. Jedyny neutralny element: bardzo duza liczba waskich wpisow blogowych (SEO long-tail).</t>
+        </is>
+      </c>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>Zakres tematyczny zgodny z poprzednim opisem, ale POMINIETO brak uprawnien zawodowych wlasciciela i watpliwy etycznie model biznesowy (skup zadluzonych spolek).</t>
+        </is>
+      </c>
+      <c r="M4" s="13" t="inlineStr">
+        <is>
+          <t>Bardzo duży wolumen treści SEO (dziesiątki wpisów o 299/586 KSH, ZUS, US, komornikach), rozbudowana oferta produktowa (sklep z gotowymi usługami).</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
+          <t>Brak tytułu zawodowego prowadzącego (nie radca prawny, nie adwokat), kontrowersyjny etycznie model biznesowy oparty głównie o "skup zadłużonych spółek", brak cen na stronie.</t>
+        </is>
+      </c>
+      <c r="O4" s="13" t="inlineStr">
+        <is>
+          <t>KRS Guard może podkreślać uprawnienia zawodowe (radca prawny) i przejrzysty, etyczny model jako kontrast wobec tej konkurencji — silny argument wiarygodności.</t>
+        </is>
+      </c>
+      <c r="P4" s="13" t="inlineStr">
+        <is>
+          <t>Duży wolumen treści SEO może zabierać ruch na frazy ogólne o art. 299 KSH mimo wątpliwej wiarygodności biznesowej firmy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Sieńko Pięta i Partnerzy</t>
@@ -886,7 +1067,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Dedykowana usługa "Ochrona Członków Zarządu": art. 299, D&amp;O, upadłość/restrukturyzacja</t>
+          <t>Potwierdzone w pelni: obszerna (24 min czytania) dedykowana podstrona "Ochrona Czlonkow Zarzadu" (sienkoipartnerzy.pl/zakres-uslug/ochrona-czlonkow-zarzadu/). Cytat: "jezeli egzekucja przeciwko spolce okaze sie bezskuteczna, wierzyciel (np. kontrahent, urzad skarbowy, ZUS) moze skierowac pozew z art. 299 k.s.h. bezposrednio przeciwko Tobie." Osobne sekcje: art. 299 KSH, upadlosc/restrukturyzacja, doradztwo D&amp;O, FAQ.</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -909,8 +1090,48 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="60" customHeight="1">
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>CZESCIOWO - partnerzy zarzadzajacy (Sienko, Pieta) to ADWOKACI; w zespole jest jeden radca prawny (Marcin Talma), ale nie jest partnerem/zalozycielem.</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>Brak cytowanych, imiennych opinii klientow - tylko ogolne deklaracje wartosci (dyskrecja, zaufanie).</t>
+        </is>
+      </c>
+      <c r="K5" s="13" t="inlineStr">
+        <is>
+          <t>FAQ wbudowane bezposrednio w podstrone uslugi (nie osobno), odpowiadajace na konkretne obawy klienta - dobry wzorzec do skopiowania na Cenniku/podstronie uslug KRS Guard.</t>
+        </is>
+      </c>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>W PELNI ZGODNY z poprzednim opisem, potwierdzony zrodlowo.</t>
+        </is>
+      </c>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t>Najbardziej dopracowana merytorycznie podstrona usługowa w całej grupie (art. 299 + D&amp;O + upadłość/restrukturyzacja w jednym miejscu), dobre FAQ wbudowane bezpośrednio w usługę.</t>
+        </is>
+      </c>
+      <c r="N5" s="13" t="inlineStr">
+        <is>
+          <t>Brak cen na stronie, brak jawnych, imiennych opinii klientów, model głównie stacjonarny z opcją zdalną (nie w pełni zdalnie jak KRS Guard).</t>
+        </is>
+      </c>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t>Brak transparentnego cennika — KRS Guard może kontrastować jawną ceną Audytu 48h "od 900 zł" jako rzadkość na rynku.</t>
+        </is>
+      </c>
+      <c r="P5" s="13" t="inlineStr">
+        <is>
+          <t>Jedna z najbardziej kompletnych merytorycznie ofert w Tier 1 — realne ryzyko przegranej walki o frazę "ochrona członków zarządu" w wyszukiwarce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Kłodziński Kancelaria (Piotr Kłodziński)</t>
@@ -928,7 +1149,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Wyspecjalizowana wyłącznie w obronie z art. 299 KSH, strategia oparta o wyrok TK P 5/19</t>
+          <t>Dedykowany, bardzo obszerny (19 min) artykul "Pozew z art. 299 KSH - jak skutecznie bronic czlonka zarzadu?" z sekcja o wyroku TK P 5/19. ALE: firma NIE jest wyspecjalizowana wylacznie w art. 299 KSH - to ogolna kancelaria warszawsko-krakowska z ok. 10 obszarami praktyki (prawo farmaceutyczne, najem nieruchomosci komercyjnych, prawo pracy, rodzinne, cywilne). Art. 299 to jeden punkt z wielu, nie wylaczna specjalizacja.</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -951,8 +1172,48 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="60" customHeight="1">
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>TAK - Piotr Klodzinski, Radca Prawny, Zalozyciel Kancelarii (potwierdzone na stronie glownej i w stopce artykulu).</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>TAK - jedyna z tej grupy z realnymi, imiennymi testimonialami ze zdjeciami i rolami (np. Anna Gorska, specjalista ds. marketingu: "Widac doswiadczenie korporacyjne - Pan Mecenas zawsze pokazuje wszystkie ryzyka i druga strone medalu [...]").</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>(a) Imienne opinie z rola/firma klienta zamiast anonimowych gwiazdek - silnie buduje zaufanie; (b) stale, zryczaltowane ceny publikowane wprost ("Gwarancja stalej ceny").</t>
+        </is>
+      </c>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>ZNACZACO PRZESADZONY: nie jest wyspecjalizowana wylacznie w art. 299 KSH, to butikowa, ale ogolna kancelaria z jedna dobra nisza. Watek wyroku TK P 5/19 - trafny i potwierdzony.</t>
+        </is>
+      </c>
+      <c r="M6" s="13" t="inlineStr">
+        <is>
+          <t>Realne, imienne opinie klientów ze zdjęciami i rolami (jedyna taka w tej grupie), stałe, zryczałtowane ceny publikowane wprost ("Gwarancja stałej ceny"), radca prawny na czele.</t>
+        </is>
+      </c>
+      <c r="N6" s="13" t="inlineStr">
+        <is>
+          <t>Nie jest wyspecjalizowana wyłącznie w temacie — ochrona zarządu to jeden z ok. 10 obszarów praktyki (farmaceutyczne, najem, prawo pracy, rodzinne) — może rozmywać przekaz wobec klienta szukającego wąskiego specjalisty.</t>
+        </is>
+      </c>
+      <c r="O6" s="13" t="inlineStr">
+        <is>
+          <t>KRS Guard jako WĄSKI, jednotematyczny specjalista (nie jeden z wielu obszarów) może kontrastować z ich rozproszoną, ogólną ofertą.</t>
+        </is>
+      </c>
+      <c r="P6" s="13" t="inlineStr">
+        <is>
+          <t>Silny, konkretny dowód społeczny (imienne opinie z rolą/firmą klienta) może przeważać u klienta mimo węższej specjalizacji tej kancelarii w temacie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="150" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Be Law</t>
@@ -970,7 +1231,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Dedykowana podstrona obrony z art. 299 + osobny materiał o ZUS/podatkach</t>
+          <t>Potwierdzone w pelni: dedykowana podstrona uslugi "Odpowiedzialnosc zarzadu" (belaw.pl/uslugi/odpowiedzialnosc-zarzadu/) + swiezy (17.07.2026) artykul blogowy z FAQ i linkiem do osobnego materialu o ZUS/podatkach (belaw.pl/czlonek-zarzadu-zus-podatki/).</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -993,8 +1254,48 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>TAK - czterech partnerow zarzadzajacych, wszyscy tytulowani "radca prawny" z numerami wpisu OIRP (Orlinska, Chamier-Gliszczynski, Jakubowski, Polanski).</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>Naglowek "co mowia o nas klienci" istnieje na stronie glownej, ale tresc nie zostala przechwycona (prawdopodobnie widget JS/karuzela) - wymaga sprawdzenia wizualnego w przegladarce, niepotwierdzone.</t>
+        </is>
+      </c>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>Swieze, regularnie publikowane artykuly blogowe w formule Q&amp;A z FAQ na koncu - dobry wzorzec do SEO i realnej wartosci dla czytelnika.</t>
+        </is>
+      </c>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>POTWIERDZONY WIERNIE, z konkretnym adresem URL i trescia zgodna z zapowiedzia.</t>
+        </is>
+      </c>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t>Czterech radców prawnych na czele (jawne numery OIRP), świeże, regularnie publikowane artykuły w formule Q&amp;A z FAQ, dedykowana usługa + osobny materiał o ZUS/podatkach.</t>
+        </is>
+      </c>
+      <c r="N7" s="13" t="inlineStr">
+        <is>
+          <t>Brak potwierdzonych opinii klientów na stronie, wyłącznie/głównie stacjonarnie (Bydgoszcz), brak cen na stronie.</t>
+        </is>
+      </c>
+      <c r="O7" s="13" t="inlineStr">
+        <is>
+          <t>Brak jawnego cennika i modelu zdalnego — przewaga dla KRS Guard w komunikacji.</t>
+        </is>
+      </c>
+      <c r="P7" s="13" t="inlineStr">
+        <is>
+          <t>Duży, wiarygodny zespół radców prawnych + świeży, regularny content = realna konkurencja SEO właśnie na frazy ZUS/US, które plan marketingowy KRS Guard wskazuje jako priorytetową szansę.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="150" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Dowlegal (Decowska-Olejnik)</t>
@@ -1012,7 +1313,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Partner zarządzający opisywany wprost jako "obrońca interesów członków zarządu"</t>
+          <t>Dedykowana podstrona specjalizacji (dowlegal.pl/nasze-specjalizacje/odpowiedzialnosc-czlonkow-zarzadu/): odpowiedzialnosc cywilna/karna/finansowa, subsydiarna, spory z ZUS i US, D&amp;O, restrukturyzacje, 11-punktowe FAQ.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -1035,8 +1336,48 @@
           <t>300+ spraw wygranych / 500+ klientów (ogólne)</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>NIE - kancelaria adwokacka. Oboje zalozyciele to adwokaci (Julia Decowska-Olejnik, Rafal Olejnik), Izba Adwokacka w Warszawie.</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>TAK, ok. 10 pelnych, podpisanych opinii na /o-nas/ - ALE wszystkie dotycza spraw FRANKOWYCH (CHF), zadna nie odnosi sie do odpowiedzialnosci zarzadu.</t>
+        </is>
+      </c>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>Osobny "Kalkulator sankcji" (dla frankowiczow) w menu glownym obok CTA "Bezplatna analiza" - struktura lejka bardzo podobna do KRS Guard (kalkulator -&gt; bezplatna analiza -&gt; usluga).</t>
+        </is>
+      </c>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>CZESCIOWA NIESCISLOSC: dedykowany cytat "obronca interesow czlonkow zarzadu" NIE istnieje dosownie - to parafraza zblizonego znaczeniowo zdania z bio prawnika. Tresc merytoryczna oferty potwierdzona.</t>
+        </is>
+      </c>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>Liczne, realne, podpisane opinie klientów (choć głównie ze spraw frankowych), własny działający "Kalkulator sankcji" pokazujący doświadczenie w budowie podobnych narzędzi lejkowych, bezpłatna analiza jako pierwszy krok.</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="inlineStr">
+        <is>
+          <t>Kancelaria adwokacka (nie radcowska), temat ochrony zarządu to poboczna specjalizacja (główny profil firmy to sprawy frankowe), zero opinii dotyczących konkretnie tematu zarządu.</t>
+        </is>
+      </c>
+      <c r="O8" s="13" t="inlineStr">
+        <is>
+          <t>Brak realnych opinii specyficznie o ochronie zarządu — KRS Guard może budować i eksponować opinie dotyczące dokładnie tego tematu jako przewagę wiarygodności.</t>
+        </is>
+      </c>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>Firma ma już sprawny, działający lejek z kalkulatorem (dla innego tematu) — realne ryzyko, że szybko zbuduje analogiczne narzędzie dla ochrony zarządu, gdyby uznała temat za priorytetowy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="150" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Staniek&amp;Partners</t>
@@ -1054,7 +1395,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>"Chronimy członków zarządu" — analiza ryzyka, D&amp;O, szkolenia dla kadry</t>
+          <t>W pelni potwierdzone, niemal doslowny naglowek strony: "Chronimy czlonkow zarzadu przed ryzykiem odpowiedzialnosci osobistej i karnej" (staniekandpartners.pl/prawo/odpowiedzialnosc-czlonkow-zarzadu/). Osobna, rownolegla podstrona "Ochrona kadry zarzadzajacej D&amp;O".</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -1077,8 +1418,48 @@
           <t>100+ wygranych sporów / 300 klientów (ogólne)</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="60" customHeight="1">
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>TAK - dr Krzysztof Staniek, wspolzalozyciel, "Radca prawny i licencjonowany doradca podatkowy" (+ doktorat nauk prawnych).</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>Brak klasycznych opinii tekstowych - sekcja "Te firmy nam zaufaly" (loga: Sokolow S.A., Deichmann, Fakro) + podstrona "Rekomendacje" z pojedynczymi wpisami nazwanymi po kliencie, ale tresci samych listow nie udalo sie odczytac (prawdopodobnie skan/grafika).</t>
+        </is>
+      </c>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>Rozdzielenie na dwie uslugi (ochrona ogolna vs. konkretnie ubezpieczenie D&amp;O) to sensowna segmentacja oferty; FAQ wbudowane bezposrednio w strone uslugi.</t>
+        </is>
+      </c>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>POTWIERDZONY NIEMAL DOSLOWNIE, laczenie z konkretnymi sformulowaniami z naglowka strony.</t>
+        </is>
+      </c>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>Bardzo precyzyjnie nazwana, kompletna oferta (dosłowny nagłówek "Chronimy członków zarządu"), osobna usługa D&amp;O, duzi, rozpoznawalni klienci referencyjni (Sokołów S.A., Deichmann, Fakro), radca prawny + doradca podatkowy na czele, obecność w 4 miastach.</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="inlineStr">
+        <is>
+          <t>Wyłącznie/głównie stacjonarnie (4 fizyczne biura, brak modelu zdalnego), brak cen na stronie, brak czytelnych opinii tekstowych (tylko logotypy i niedostępne "Rekomendacje").</t>
+        </is>
+      </c>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t>Brak przejrzystego cennika i modelu zdalnego — jeden z mocniejszych kontrastów do wykorzystania w komunikacji KRS Guard.</t>
+        </is>
+      </c>
+      <c r="P9" s="13" t="inlineStr">
+        <is>
+          <t>NAJBLIŻSZY tematycznie i wizerunkowo konkurent w całym Tier 1 — kompletna, precyzyjnie nazwana oferta plus duzi klienci referencyjni budują bardzo silną wiarygodność.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="150" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>PLA.partners</t>
@@ -1096,7 +1477,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Dedykowana podstrona o art. 299 KSH; wsparcie dla pozwanych i wierzycieli</t>
+          <t>Brak stalej pozycji w menu uslug (w nawigacji jest ogolniejsza "Ochrona majatku"), ale jest dedykowany, obszerny (7 min) ARTYKUL BLOGOWY wylacznie o tym temacie (pla.partners/odpowiedzialnosc-na-gruncie-art-299-ksh/). Cytat: "Nasz zespol wspomaga nie tylko wierzycieli w dochodzeniu roszczen na podstawie art. 299 KSH, ale oferuje rowniez przedsiebiorcom [czlonkom zarzadu] pomoc prawna..."</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1119,8 +1500,48 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>CZESCIOWO - zalozyciel Maciej Pilarek to ADWOKAT, nie radca prawny; wspolzalozycielka Paulina Lubas ma tytul LL.M. (bez polskiego tytulu zawodowego). Radcowie prawni sa w zespole, ale nie na czele.</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>Brak - tylko siatka logotypow firm-klientow ("Zaufali nam"), bez cytowanych opinii tekstowych.</t>
+        </is>
+      </c>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>Wewnetrzne linkowanie SEO: na koncu artykulu lista 13 linkowanych uslug powiazanych, kazda z fraza kluczowa typu "odpowiedzialnosc czlonka zarzadu radca prawny" - dlugi ogon fraz.</t>
+        </is>
+      </c>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>DROBNA NIESCISLOSC: to nie "dedykowana podstrona" w stalym menu, tylko artykul blogowy (funkcjonalnie zblizony). Tresc merytoryczna ("wsparcie dla pozwanych i wierzycieli") potwierdzona w pelni.</t>
+        </is>
+      </c>
+      <c r="M10" s="13" t="inlineStr">
+        <is>
+          <t>Wsparcie obu stron sporu (szerszy potencjalny rynek), dobre wewnętrzne linkowanie SEO z długim ogonem fraz, obecność radców prawnych w zespole.</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="inlineStr">
+        <is>
+          <t>Osoba na czele to adwokat, nie radca prawny; brak opinii klientów; temat funkcjonuje jako artykuł blogowy, nie stała, wyeksponowana usługa w menu.</t>
+        </is>
+      </c>
+      <c r="O10" s="13" t="inlineStr">
+        <is>
+          <t>Brak stałej pozycji tematu w menu usług — sygnał, że nie jest dla nich priorytetowy; KRS Guard może wygrywać widocznością i pozycjonowaniem tematu jako głównego, jedynego produktu.</t>
+        </is>
+      </c>
+      <c r="P10" s="13" t="inlineStr">
+        <is>
+          <t>Niskie/średnie — temat wygląda na poboczny wątek szerszej praktyki gospodarczej firmy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="150" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>KSK (Kosmus i Łojkowska Radcy Prawni)</t>
@@ -1138,7 +1559,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Wsparcie prawne w sporach z art. 299 + doradztwo D&amp;O</t>
+          <t>Potwierdzone: wpis blogowy "Odpowiedzialnosc czlonka zarzadu za dlugi spolki, czyli art. 299 KSH w praktyce" (autor: r.pr. Aleksander Kosmus, 22.07.2026) + osobna, rozbudowana podstrona uslugowa "Sprawy sadowe na tle ubezpieczen D&amp;O" (likwidacja szkod D&amp;O, obrona przy odmowie wyplaty, analiza OWU).</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1161,8 +1582,48 @@
           <t>27 000+ spraw / 1000+ klientów (ogólne)</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="60" customHeight="1">
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>TAK - oboje zalozyciele: Aleksander Kosmus ("Radca prawny, Partner Zalozyciel") i Joanna Lojkowska ("Radca prawna, Partnerka zarzadzajaca"). Zespol: 5 radcow prawnych + 3 adwokatow.</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>Brak cytowanych opinii/case studies - tylko zbiorcze liczby ("1000+ klientow", "27000+ spraw", "300 mln zl wartosci roszczen") bez konkretnych referencji.</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>Osobna, konkretna oferta D&amp;O jako komplementarny temat do art. 299 KSH - warto rozwazyc wzmianke o D&amp;O jako uzupelnieniu ochrony zarzadu. FAQ przy artykule blogowym odpowiadajace na konkretne pytania praktyczne.</t>
+        </is>
+      </c>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>W PELNI POTWIERDZONY - jeden z najbardziej rzetelnych opisow w calym zestawieniu, oba elementy (art. 299 + D&amp;O) realne i dobrze udokumentowane.</t>
+        </is>
+      </c>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t>Oboje założyciele to radcowie prawni, bardzo duży, udokumentowany ogólny dorobek (27000+ spraw, 1000+ klientów), osobna, rozbudowana oferta D&amp;O jako komplementarny temat, artykuł z FAQ praktycznym.</t>
+        </is>
+      </c>
+      <c r="N11" s="13" t="inlineStr">
+        <is>
+          <t>Brak imiennych opinii/case studies (tylko zbiorcze liczby), wyłącznie/głównie stacjonarnie (Gdańsk), konsultacja PŁATNA (400-600 zł) — brak darmowego pierwszego kroku.</t>
+        </is>
+      </c>
+      <c r="O11" s="13" t="inlineStr">
+        <is>
+          <t>Płatna konsultacja i brak modelu zdalnego — bezpośrednia przewaga dla darmowego Kalkulatora ryzyka i pracy zdalnej w całej Polsce oferowanych przez KRS Guard.</t>
+        </is>
+      </c>
+      <c r="P11" s="13" t="inlineStr">
+        <is>
+          <t>Bardzo duże ogólne doświadczenie firmy (27000+ spraw) i uzupełniający temat D&amp;O mogą budować przewagę wizerunkową mimo braku liczb specyficznych dla ochrony zarządu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="150" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>UpStart Legal</t>
@@ -1180,7 +1641,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Niemal wyłącznie ten temat: analiza ryzyka, strategia obrony, ochrona majątku prywatnego</t>
+          <t>Dedykowana podstrona "Odpowiedzialnosc czlonkow zarzadu (art. 299 k.s.h.) - Katowice, Slask" z 4 blokami (analiza ryzyka, strategia dzialania, obrona w sporach, ochrona majatku prywatnego) - potwierdza opis. ALE to jedna z SZESCIU rownorzednych uslug firmy (obok upadlosci konsumenckiej, ktora dominuje strone glowna); nie "niemal wylacznie ten temat".</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1203,8 +1664,48 @@
           <t>50+ spraw / 30+ klientów (ogólne)</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="60" customHeight="1">
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>NIE JAWNIE - zalozyciel Lukasz Cieslik opisany jako "prawnik z ponad osmioletnim doswiadczeniem", bez tytulu radcy/adwokata. W zespole jest wymieniona z nazwiska Adwokat Paulina Stepien.</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>Tylko zbiorcze liczniki (50+ ukonczonych spraw, 30+ zadowolonych klientow, +30 pozytywnych opinii) bez wyswietlonej tresci - zadnych cytowanych, indywidualnych opinii.</t>
+        </is>
+      </c>
+      <c r="K12" s="13" t="inlineStr">
+        <is>
+          <t>Jawny, rozpisany cennik (4 warianty od najtanszego do pelnej obslugi) - rzadkosc w branzy, buduje zaufanie; "Sprawdz swoja zdolnosc upadlosciowa" jako lead magnet podobny mechanizmem do Kalkulatora ryzyka KRS Guard.</t>
+        </is>
+      </c>
+      <c r="L12" s="13" t="inlineStr">
+        <is>
+          <t>CZESCIOWO ZAWYZONE: cennik (150 zl konsultacja / 500 zl sprawdzenie wniosku / od 5500 zl pelna obsluga) potwierdzony aktualny, ALE dotyczy uslugi upadlosci konsumenckiej, nie osobno wycenionej ochrony zarzadu - laczenie mylace. "Niemal wylacznie ten temat" - przesadzone, to 1 z 6 rownorzednych uslug.</t>
+        </is>
+      </c>
+      <c r="M12" s="13" t="inlineStr">
+        <is>
+          <t>JEDYNA firma w Tier 1 działająca wyłącznie zdalnie (jak KRS Guard), jawny, rozpisany cennik (4 warianty), lead magnet "sprawdź swoją zdolność upadłościową".</t>
+        </is>
+      </c>
+      <c r="N12" s="13" t="inlineStr">
+        <is>
+          <t>Temat ochrony zarządu to 1 z 6 równorzędnych usług (nie priorytet firmy — dominuje upadłość konsumencka), założyciel bez jawnie podanego tytułu zawodowego, brak liczb specyficznych dla tematu zarządu.</t>
+        </is>
+      </c>
+      <c r="O12" s="13" t="inlineStr">
+        <is>
+          <t>Temat nie jest ich głównym produktem, tylko jednym z sześciu — KRS Guard może wygrywać pełnym skupieniem WYŁĄCZNIE na ochronie zarządu zamiast bycia jedną z wielu usług.</t>
+        </is>
+      </c>
+      <c r="P12" s="13" t="inlineStr">
+        <is>
+          <t>JEDYNY realny konkurent z tym samym modelem obsługi (wyłącznie zdalnie) i podobnym podejściem do jawności cen — warto obserwować, czy nie rozwinie mocniej właśnie tego tematu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="150" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Kancelaria Tyrka (Marta Tyrka)</t>
@@ -1222,7 +1723,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Udokumentowane realnie wygrane sprawy z art. 299 KSH</t>
+          <t>Wpis "Odpowiedzialnosc czlonka zarzadu" z 21.08.2020 - NIEAKTUALIZOWANY od tego czasu, poza glownym menu (dostepny tylko przez wyszukiwarke). Jedno zdanie o wlasnych sprawach: "W sprawach prowadzonych przez Kancelarie udalo sie wygrac kilka procesow prowadzonych w imieniu czlonkow zarzadu dzieki wykazaniu przeslanki nr 3."</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1245,8 +1746,48 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="60" customHeight="1">
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>TAK - Marta Tyrka, "radca prawny oraz staly mediator sadowy" (OIRP Szczecin nr SZ-1344).</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>Zakladka "Zaufali" w nawigacji sugeruje sekcje z referencjami, ale niezweryfikowana (strona zbyt duza do pelnego pobrania) - do sprawdzenia recznie.</t>
+        </is>
+      </c>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>Infografika "jak przebiega standardowa droga do otrzymania pozwu z art. 299 ksh" - prosty, latwy do adaptacji format edukacyjny (wizualizacja sciezki od bezskutecznej egzekucji do pozwu).</t>
+        </is>
+      </c>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>PRZESADZONY: "udokumentowane realnie wygrane sprawy" to w rzeczywistosci jedno ogolne zdanie BEZ zadnej dokumentacji (sygnatur, dat, opisu stanu faktycznego) na nieaktualizowanym od 2020 r. wpisie blogowym.</t>
+        </is>
+      </c>
+      <c r="M13" s="13" t="inlineStr">
+        <is>
+          <t>Radca prawny prowadząca, deklarowane doświadczenie w sprawach z art. 299 KSH.</t>
+        </is>
+      </c>
+      <c r="N13" s="13" t="inlineStr">
+        <is>
+          <t>Treść nieaktualizowana od 2020 r., poza głównym menu strony (dostępna tylko przez wyszukiwarkę), brak jakiejkolwiek dokumentacji "wygranych spraw" (sygnatur, dat, opisu), niejasna płatność za porady online.</t>
+        </is>
+      </c>
+      <c r="O13" s="13" t="inlineStr">
+        <is>
+          <t>Bardzo słaby, zaniedbany konkurent na tym froncie — niska bariera do wyprzedzenia w SEO i wiarygodności treści.</t>
+        </is>
+      </c>
+      <c r="P13" s="13" t="inlineStr">
+        <is>
+          <t>Minimalne.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="150" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Wardyn Doradztwo Restrukturyzacyjne</t>
@@ -1264,7 +1805,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Wyspecjalizowana w obronie członków zarządu przed odpowiedzialnością materialną</t>
+          <t>Dedykowana podstrona w glownym menu "Ochrona czlonkow zarzadu". Cytat: "bronimy czlonkow zarzadow przed odpowiedzialnoscia materialna za zobowiazania spolki, ktora reprezentowali. Jestesmy w stanie zgromadzic szeroki i rzetelny material dowodowy..." Rozroznia odpowiedzialnosc cywilnoprawna (specjalizacja wlasna) od karnej (tu wspolpraca z zewnetrznym adwokatem).</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1287,8 +1828,48 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="60" customHeight="1">
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>NIE - to doradcy restrukturyzacyjni, nie kancelaria radcowska/adwokacka. Przemyslaw Wardyn: "Ekonomista, Licencjonowany Doradca Restrukturyzacyjny"; Mateusz Wardyn: "Prawnik, Licencjonowany Doradca Restrukturyzacyjny" - tytul "Prawnik", NIE radca prawny/adwokat.</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>TAK, realne - sekcja "Opinie o nas" zintegrowana z Google (5.0 na podstawie 27 opinii). Cytat od Prezesa Zarzadu klienta: "Dla mnie jako czlonka zarzadu spolki przechodzacej przez restrukturyzacje ich fachowa pomoc byla nieoceniona."</t>
+        </is>
+      </c>
+      <c r="K14" s="13" t="inlineStr">
+        <is>
+          <t>Realne opinie zintegrowane z Google, w tym jedna z perspektywy prezesa zarzadu w restrukturyzacji - bardzo trafny social proof dla dokladnie naszej grupy docelowej.</t>
+        </is>
+      </c>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>TRESCIOWO POTWIERDZONY, ale POMINIETY kluczowy fakt: to firma doradztwa restrukturyzacyjnego prowadzona przez licencjonowanych doradcow restrukturyzacyjnych, NIE kancelaria radcy prawnego/adwokacka - inny profil zawodowy niz sugerowalaby nazwa "Kancelaria".</t>
+        </is>
+      </c>
+      <c r="M14" s="13" t="inlineStr">
+        <is>
+          <t>Realne, zintegrowane z Google opinie (5.0 z 27 opinii), w tym trafna opinia od prezesa zarządu klienta w restrukturyzacji — bardzo mocny, wiarygodny social proof dla dokładnie tej grupy docelowej; dedykowana podstrona w głównym menu.</t>
+        </is>
+      </c>
+      <c r="N14" s="13" t="inlineStr">
+        <is>
+          <t>To NIE kancelaria prawna — prowadzona przez licencjonowanych doradców restrukturyzacyjnych bez tytułu radcy prawnego/adwokata, co może budzić wątpliwości u klienta szukającego prawnika; obsługa spraw karnych zlecana na zewnątrz (współpraca z zewnętrznym adwokatem).</t>
+        </is>
+      </c>
+      <c r="O14" s="13" t="inlineStr">
+        <is>
+          <t>KRS Guard (radca prawny na czele, pełne uprawnienia prawnicze) może wprost kontrastować brak uprawnień prawniczych tej firmy — mocny argument wiarygodności.</t>
+        </is>
+      </c>
+      <c r="P14" s="13" t="inlineStr">
+        <is>
+          <t>Bardzo dobre, realne opinie klientów trafiające dokładnie w naszą grupę docelową (członek zarządu w restrukturyzacji) — trudny do szybkiego skopiowania dowód społeczny.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="150" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>M.D. Legal Solutions (Monika Drab)</t>
@@ -1306,7 +1887,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Cała marka poświęcona temu tematowi; model: abonament doradczy + szkolenia + podcast, BEZ kalkulatora/pakietów</t>
+          <t>Cala domena to marka poswiecona wylacznie temu tematowi. Kluczowa usluga: platny Abonament "Odpowiedzialnosc Czlonka Zarzadu" (model "mowisz i masz" - doradca dostepny na biezaco), plus sklep z dokumentami/uslugami, platforma szkolen VOD i podcast "Prawne sekrety zarzadow spolek". Brak kalkulatora i brak "pakietow" w rozumieniu KRS Guard.</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1329,8 +1910,48 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>TAK - Monika Drab, radczyni prawna (jawnie wielokrotnie na stronie) + licencjonowana doradczyni restrukturyzacyjna (nr 1616) + ekspertka BCC, 20+ lat doswiadczenia.</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>Brak - tylko "Najnowsze komentarze" czytelnikow pod wpisami blogowymi, nie referencje klientow uslugi.</t>
+        </is>
+      </c>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>Model abonamentowy "doradca na telefon, zanim problem sie zmaterializuje" - ciekawa alternatywa dla podejscia "reaguj po fakcie". Podcast + VOD to duzy naklad pracy, niekoniecznie do skopiowania wprost.</t>
+        </is>
+      </c>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>ZGADZA SIE W PELNI z poprzednim opisem.</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="inlineStr">
+        <is>
+          <t>Cała marka wyłącznie o tym temacie, radczyni prawna z 20+ lat doświadczenia, rozbudowany content (podcast, platforma VOD), model abonamentowy prewencyjny ("doradca na telefon zanim problem się zmaterializuje").</t>
+        </is>
+      </c>
+      <c r="N15" s="13" t="inlineStr">
+        <is>
+          <t>Brak kalkulatora i brak pakietów, brak jawnych opinii klientów, ceny głównego abonamentu niejawne, działalność wygląda na jednoosobową (brak widocznego zespołu/skalowalności).</t>
+        </is>
+      </c>
+      <c r="O15" s="13" t="inlineStr">
+        <is>
+          <t>Brak transparentnego cennika głównej usługi i brak kalkulatora ryzyka — bezpośrednia, łatwa do komunikowania przewaga KRS Guard.</t>
+        </is>
+      </c>
+      <c r="P15" s="13" t="inlineStr">
+        <is>
+          <t>Najbardziej wyspecjalizowana marka na rynku obok KRS Guard (cała domena poświęcona wyłącznie temu tematowi) — realne ryzyko konkurowania o te same, wąskie frazy kluczowe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="150" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Jakubowska-Zawada</t>
@@ -1348,7 +1969,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Dedykowana usługa: analiza ryzyka transakcji, strategia obrony, bezpieczne zakończenie mandatu</t>
+          <t>Dedykowana podstrona "Ochrona Czlonkow Zarzadu" (meta: "Ochrona Czlonkow Zarzadu - Adwokat | art. 299 KSH, NIS2"): obrona przed odpowiedzialnoscia cywilna (art. 299 KSH), karna, karno-skarbowa, administracyjna, plus nowosc - NIS2/cyberbezpieczenstwo od 3.04.2026.</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1371,8 +1992,48 @@
           <t>1000+ spraw (ogólne)</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="60" customHeight="1">
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>NIE - Joanna Jakubowska-Zawada, ADWOKAT (nie radca prawny), Okregowa Rada Adwokacka w Rzeszowie od 2010 r., wlascicielka kancelarii.</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
+        <is>
+          <t>Tylko zbiorcze statystyki ("99% zadowolonych klientow", "1000+ spraw", "300 mln+ PLN") - brak pojedynczych cytowanych opinii z nazwiskiem.</t>
+        </is>
+      </c>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>Krotkie "W skrocie" podsumowanie na gorze kazdej podstrony uslugowej (2-3 zdania przed pelnym tekstem) - dobry wzorzec UX. Rozbudowane FAQ tlumaczace roznice adwokat/radca prawny/kancelaria odszkodowawcza.</t>
+        </is>
+      </c>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>W WIEKSZOSCI ZGODNY - "analiza ryzyka" i "strategia obrony" sa doslownie na stronie. Element "bezpieczne zakonczenie mandatu" nie wystepuje wprost na sprawdzonej podstronie (moglo byc interpretacja ogolnego zakresu uslug).</t>
+        </is>
+      </c>
+      <c r="M16" s="13" t="inlineStr">
+        <is>
+          <t>Szeroki zakres tematyczny (cywilna/karna/karno-skarbowa/administracyjna + nowość NIS2/cyberbezpieczeństwo), dobre UX (podsumowanie "W skrócie" na górze strony), FAQ tłumaczące różnicę adwokat/radca prawny.</t>
+        </is>
+      </c>
+      <c r="N16" s="13" t="inlineStr">
+        <is>
+          <t>Adwokat, nie radca prawny; brak imiennych opinii klientów (tylko zbiorcze statystyki); brak cen na stronie.</t>
+        </is>
+      </c>
+      <c r="O16" s="13" t="inlineStr">
+        <is>
+          <t>Brak cen i brak modelu zdalnego (Rzeszów, stacjonarnie) — kolejny przykład przewagi cenowej i modelowej KRS Guard do wykorzystania w komunikacji.</t>
+        </is>
+      </c>
+      <c r="P16" s="13" t="inlineStr">
+        <is>
+          <t>Aktywnie rozwijana, aktualizowana oferta (dodają nawet nowy temat NIS2) — realna, żywa konkurencja, nie zaniedbana strona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="150" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>PW Restrukturyzacja</t>
@@ -1390,7 +2051,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Ochrona majątku prywatnego członków zarządu przy zagrożeniu niewypłacalnością</t>
+          <t>Dedykowana podstrona uslugi "Ochrona czlonkow zarzadu w spolkach" (naglowek "Zabezpieczenie majatku czlonka zarzadu"): "Zapewniamy ochrone majatku czlonkow zarzadow w spolkach, ktore sa zagrozone niewyplacalnoscia lub sa w stanie niewyplacalnosci. Reprezentujemy czlonkow zarzadu w sporach z wierzycielami." Proces w 6 krokach + osobny artykul o art. 299 KSH i art. 116 Ordynacji podatkowej.</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1413,8 +2074,48 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="60" customHeight="1">
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>TAK - Krzysztof Piotrowski (Radca Prawny, Kwalifikowany Doradca Restrukturyzacyjny, Mediator Sadowy) i Krzysztof Proc (Radca Prawny, Doradca Restrukturyzacyjny, Dyrektor Dzialu Prawnego).</t>
+        </is>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>TAK - 5 nazwanych recenzji 5-gwiazdkowych na stronie glownej (Magdalena Klebek-Wielgo, Marcin Atkaczunas, Krzysztof Guzowski, Dominik Liszewski, Celina Soltys).</t>
+        </is>
+      </c>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>Case studies z konkretnymi liczbami ("Suma korzysci dla klienta: 291 734 zl", "Czas realizacji: 83 dni") - bardzo przekonujacy format social proof, wart skopiowania. Artykul-"test" ("Kiedy ryzykujesz prywatnym majatkiem? [Test]") jako format angazujacy.</t>
+        </is>
+      </c>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>ZGADZA SIE W PELNI - najbardziej solidnie potwierdzony wpis w calym zestawieniu (dedykowana usluga + realne opinie + radcowie prawni jawnie wskazani).</t>
+        </is>
+      </c>
+      <c r="M17" s="13" t="inlineStr">
+        <is>
+          <t>NAJLEPIEJ potwierdzony wpis w całym zestawieniu: dedykowana usługa w menu, realne imienne opinie 5-gwiazdkowe, case studies z konkretnymi liczbami (kwoty korzyści, czas realizacji), radcowie prawni na czele, jasno opisany proces w 6 krokach.</t>
+        </is>
+      </c>
+      <c r="N17" s="13" t="inlineStr">
+        <is>
+          <t>Wyłącznie/głównie stacjonarnie (Warszawa), brak cen na stronie, brak modelu zdalnego.</t>
+        </is>
+      </c>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>Brak jawnego cennika i modelu zdalnego — mocny kontrast dla KRS Guard; ich case studies z konkretnymi liczbami to jednocześnie wzorzec WARTY SKOPIOWANIA na własnej stronie.</t>
+        </is>
+      </c>
+      <c r="P17" s="13" t="inlineStr">
+        <is>
+          <t>Razem ze Staniek&amp;Partners NAJSILNIEJSZY konkurent contentowo i wizerunkowo w całym zestawieniu — kompletna, w pełni potwierdzona oferta + dowód społeczny + liczbowe case studies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="150" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>KKPR / KPR Restrukturyzacja (Kaczor Madejewska)</t>
@@ -1432,7 +2133,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Kompleksowa ochrona majątku prywatnego zarządu w kryzysie + osobna podstrona o art. 116 Ordynacji podatkowej</t>
+          <t>BRAK samodzielnej, wymienionej uslugi "ochrona zarzadu" w menu (glowna oferta to restrukturyzacja/upadlosc/fundacja rodzinna). Potwierdzona dedykowana podstrona o art. 116 Ordynacji podatkowej (13 min czytania, porownanie z art. 299 KSH) oraz osobny artykul o art. 299 KSH - ale to ARTYKULY BLOGOWE (thought leadership), nie samodzielna, sprzedawana usluga widoczna w menu ofertowym.</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1455,8 +2156,48 @@
           <t>900+ postępowań (ogólne)</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="60" customHeight="1">
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>CZESCIOWO - Adam Kaczor: "adwokat i kwalifikowany doradca restrukturyzacyjny" (licencja nr 833); Ewa Madejewska: tytul "Mecenas" bez jasno podanego radca prawny/adwokat.</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>NIEPEWNE - podstrona /opinie/ istnieje z naglowkiem "Referencje i rekomendacje", ale tresc nie zostala przechwycona (prawdopodobnie widget JS) - nie potwierdzam ani obecnosci, ani braku opinii.</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>Wlasny "Kalkulator oddluzeniowy" wpiety na stale w gorne menu strony - koncepcyjnie bliskie temu, co robi KRS Guard. Mocne liczbowe wskazniki w hero ("1 miejsce 2 lata z rzedu", "83% zatwierdzonych ukladow - ponad 30% powyzej sredniej").</t>
+        </is>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>CZESCIOWO ZAWYZONY - TEN SAM TYP BLEDU CO PRZY SKARBCU: "kompleksowa ochrona majatku prywatnego" brzmi jak sprzedawana usluga, a w rzeczywistosci to glownie tresc blogowa przy glownej ofercie restrukturyzacyjnej, bez wlasnej podstrony ofertowej.</t>
+        </is>
+      </c>
+      <c r="M18" s="13" t="inlineStr">
+        <is>
+          <t>Rozpoznawalna marka restrukturyzacyjna z nagrodami ("1 miejsce 2 lata z rzędu"), własny kalkulator oddłużeniowy wbudowany na stałe w menu, mocne wskaźniki liczbowe w hero sekcji.</t>
+        </is>
+      </c>
+      <c r="N18" s="13" t="inlineStr">
+        <is>
+          <t>Brak samodzielnej, sprzedawanej usługi "ochrona zarządu" (tylko treść blogowa przy głównej ofercie restrukturyzacyjnej), niepewne opinie klientów, nie wszyscy w zespole mają jawnie podany tytuł radcy prawnego/adwokata.</t>
+        </is>
+      </c>
+      <c r="O18" s="13" t="inlineStr">
+        <is>
+          <t>Temat zarządu nie jest dla nich produktem, tylko treścią poboczną — KRS Guard może wygrywać, pozycjonując ten temat jako GŁÓWNY, samodzielny produkt zamiast dodatku do restrukturyzacji.</t>
+        </is>
+      </c>
+      <c r="P18" s="13" t="inlineStr">
+        <is>
+          <t>Mają już własny, wbudowany w menu kalkulator (inny temat) — dowód, że taki format działa w tej branży i konkurencja może go łatwo zaadaptować także dla ochrony zarządu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="150" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Worytko &amp; Słupek</t>
@@ -1474,7 +2215,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Analiza ryzyk odpowiedzialności zarządu, obrona przed roszczeniami wierzycieli</t>
+          <t>Dedykowany artykul (autor: adw. Maciej Worytko, 29.10.2025) "Odpowiedzialnosc czlonkow zarzadu w spolce z o.o. i akcyjnej - jak uniknac ryzyka osobistej odpowiedzialnosci": roznice sp. z o.o. vs S.A., obrona zarzadu (zgloszenie upadlosci w terminie), sposoby minimalizacji ryzyka (D&amp;O, dokumentacja). Konczy sie oferta: "analiza ryzyk, przygotowanie i obrona przed roszczeniami wierzycieli, postepowania upadlosciowe i restrukturyzacyjne".</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -1497,8 +2238,48 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="60" customHeight="1">
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>NIE - kancelaria adwokacka, zalozyciel adwokat Maciej Worytko.</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
+        <is>
+          <t>TAK - 3 cytowane opinie na stronie glownej (np. Pawel Horowski), ale zadna nie dotyczy spraw art. 299/zarzadu - wszystkie o innych sprawach (nieruchomosci, umowy).</t>
+        </is>
+      </c>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>Artykul podpisany imieniem i zdjeciem konkretnego prawnika (buduje autorytet); struktura "co sie dowiesz" na poczatku (jasne obietnice tresci) - prosty, tani zabieg do skopiowania.</t>
+        </is>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>POTWIERDZONY DOSLOWNIE - opis to niemal cytat z wlasnego podsumowania oferty firmy.</t>
+        </is>
+      </c>
+      <c r="M19" s="13" t="inlineStr">
+        <is>
+          <t>Artykuł podpisany imieniem i zdjęciem konkretnego prawnika (buduje autorytet), jasno opisana oferta obrony zarządu.</t>
+        </is>
+      </c>
+      <c r="N19" s="13" t="inlineStr">
+        <is>
+          <t>Adwokat, nie radca prawny; opinie na stronie nie dotyczą tematu zarządu; brak cen; mała, regionalna kancelaria (Rzeszów).</t>
+        </is>
+      </c>
+      <c r="O19" s="13" t="inlineStr">
+        <is>
+          <t>Słaby, niewyspecjalizowany konkurent na tym froncie — niska bariera do wyprzedzenia treściowo i w SEO.</t>
+        </is>
+      </c>
+      <c r="P19" s="13" t="inlineStr">
+        <is>
+          <t>Minimalne.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="150" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>KPP (Baran &amp; Pluta)</t>
@@ -1516,7 +2297,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Reprezentacja obu stron sporu (wierzyciele i zarząd) + upadłość spółek akcyjnych</t>
+          <t>Dedykowana podstrona "Odpowiedzialnosc czlonkow zarzadu Warszawa". Cytat: "Oferujemy profesjonalne doradztwo i reprezentacje zarowno dla wierzycieli, jak i czlonkow zarzadu. Niezaleznie od tego, czy potrzebuja Panstwo wsparcia w dochodzeniu roszczen, czy obronie przed nimi..."</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -1539,8 +2320,48 @@
           <t>3000+ postępowań / 2500+ likwidacji spółek (ogólne)</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="60" customHeight="1">
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>NIE JAWNIE dla zadnego z dwoch zalozycieli - Joanna Pluta (tytul niepodany), Grzegorz Baran (doradca restrukturyzacyjny i doradca podatkowy, nie radca prawny/adwokat). Trzeci wymieniony jako odpowiedzialny za ta specjalizacje, Marcin Naroznik, to ADWOKAT.</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>Brak - nie znaleziono sekcji z referencjami/testimonialami na zadnej sprawdzonej podstronie.</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>FAQ wbudowane bezposrednio w strone uslugowa; jawne rozroznienie "obslugujemy obie strony sporu" jako element transparentnosci co do konfliktu interesow.</t>
+        </is>
+      </c>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>POTWIERDZONY DOSLOWNIE - "reprezentacja obu stron sporu" to cytat ze strony.</t>
+        </is>
+      </c>
+      <c r="M20" s="13" t="inlineStr">
+        <is>
+          <t>Transparentne, jawnie skomunikowane rozróżnienie "obsługujemy obie strony sporu", FAQ wbudowane w stronę usługową, duże ogólne doświadczenie firmy (3000+ postępowań, 2500+ likwidacji spółek).</t>
+        </is>
+      </c>
+      <c r="N20" s="13" t="inlineStr">
+        <is>
+          <t>Żaden z dwóch założycieli nie jest jawnie radcą prawnym (doradca restrukturyzacyjny/podatkowy, część zespołu to adwokaci); brak opinii klientów; brak cen; obsługa obu stron sporu może budzić wątpliwości co do konfliktu interesów u klienta szukającego lojalnego obrońcy.</t>
+        </is>
+      </c>
+      <c r="O20" s="13" t="inlineStr">
+        <is>
+          <t>Brak jednoznacznych uprawnień prawniczych na czele i potencjalny konflikt interesów (obsługa obu stron) — KRS Guard może podkreślać jednoznaczne, wyłączne stanie po stronie zarządu.</t>
+        </is>
+      </c>
+      <c r="P20" s="13" t="inlineStr">
+        <is>
+          <t>Niskie/średnie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="150" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Wbrew ZUS (Kinga Matyasik-Ochlust)</t>
@@ -1558,7 +2379,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Wąsko: odwołania od decyzji ZUS o przeniesieniu odpowiedzialności na członka zarządu</t>
+          <t>Dedykowany artykul "Odpowiedzialnosc czlonka zarzadu spolki za zalegle skladki" (z 2015 r., wciaz aktywny na stronie): mechanizm art. 116 Ordynacji podatkowej stosowany odpowiednio (przez art. 31 ustawy o ub. spolecznych) do przeniesienia odpowiedzialnosci za zalegle skladki ZUS na czlonkow zarzadu, warunki obrony, krytyka praktyki ZUS przenoszenia odpowiedzialnosci tylko na wybrane osoby z zarzadu.</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1581,8 +2402,48 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="60" customHeight="1">
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>TAK - Kinga Matyasik-Ochlust, radca prawny (od 2009) + wspolpracowniczka Weronika Mania, radca prawny.</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>Brak - nie znaleziono zadnej sekcji z opiniami/referencjami.</t>
+        </is>
+      </c>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>Osobisty, nieformalny ton "O mnie" ("Kim jestem? Kobieta, matka, trzydziestolatka, radca prawnym...") - silnie buduje zaufanie. Ogromna baza blogowa (167 wpisow w samej kategorii "Odwolanie od decyzji ZUS") - buduje autorytet SEO.</t>
+        </is>
+      </c>
+      <c r="L21" s="13" t="inlineStr">
+        <is>
+          <t>TRAFNY I POTWIERDZONY, choc trzeba pamietac, ze to jeden waski watek w znacznie szerszej praktyce ZUS-owej firmy (setki innych artykulow o emeryturach, zasilkach itd.).</t>
+        </is>
+      </c>
+      <c r="M21" s="13" t="inlineStr">
+        <is>
+          <t>Radca prawny prowadząca, osobisty i autentyczny ton budujący zaufanie ("Kim jestem? Kobieta, matka, trzydziestolatka..."), ogromna baza blogowa specjalnie o ZUS (167 wpisów w samej kategorii "Odwołanie od decyzji ZUS").</t>
+        </is>
+      </c>
+      <c r="N21" s="13" t="inlineStr">
+        <is>
+          <t>Bardzo wąski zakres — wyłącznie ZUS, brak wątku art. 299 KSH i US; brak cen; brak opinii klientów; mały, dwuosobowy zespół widoczny na stronie.</t>
+        </is>
+      </c>
+      <c r="O21" s="13" t="inlineStr">
+        <is>
+          <t>Brak art. 299 KSH i US w ofercie — KRS Guard może wygrywać szerszym, zintegrowanym produktem (3 zagrożenia w 1) zamiast wąskiej specjalizacji tylko w ZUS.</t>
+        </is>
+      </c>
+      <c r="P21" s="13" t="inlineStr">
+        <is>
+          <t>REALNE zagrożenie SEO na frazy ZUS — dokładnie ta nisza, którą plan marketingowy KRS Guard wskazuje jako słabiej obsadzoną szansę, jest tu już częściowo zajęta przez dużą liczbę wpisów.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="150" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>BTLA</t>
@@ -1600,7 +2461,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Wąsko: obrona zarządu w sprawach karnych skarbowych (VAT, CIT, dotacje)</t>
+          <t>Dwie dedykowane podstrony: "Obrona zarzadu w sprawach karnych gospodarczych" i "Obrona zarzadu w sprawach karnych skarbowych" - druga z konkretnymi odwolaniami do art. 54, 56, 57, 61, 67, 80f KKS (VAT, CIT, dotacje, akcyza, MDR, nierzetelna ksiegowosc). Potwierdza waski profil - ale to jeden z wielu pionow duzej firmy doradczej (prawo + podatki + ksiegowosc + ubezpieczenia).</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1623,8 +2484,49 @@
           <t>Brak danych</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="70" customHeight="1">
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>NIE - dr Artur Oles, EMBA, "Adwokat, Doradca podatkowy, Wspolnik zarzadzajacy BTLA". Zespol karny-skarbowy zdominowany przez adwokatow i doradcow podatkowych, nie radcow prawnych.</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>Brak - jedynie puste liczniki typu "zadowolonych klientow" bez wyswietlonej wartosci w kodzie strony.</t>
+        </is>
+      </c>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>Rozbicie tematu na dwie gleboko wyspecjalizowane podstrony (gospodarcze vs skarbowe) z osobnymi FAQ i konkretnymi numerami artykulow KKS - czytelna segmentacja tematyczna. Wersje PL/EN/DE sugeruja obsluge klientow zagranicznych.</t>
+        </is>
+      </c>
+      <c r="L22" s="13" t="inlineStr">
+        <is>
+          <t>POTWIERDZONY BARDZO DOKLADNIE, wrecz z konkretnymi numerami artykulow KKS zgadzajacymi sie z opisem.</t>
+        </is>
+      </c>
+      <c r="M22" s="13" t="inlineStr">
+        <is>
+          <t>Duża, wielobranżowa firma doradcza (prawo + podatki + księgowość + ubezpieczenia), głęboka specjalizacja karno-skarbowa z konkretnymi numerami przepisów KKS, obecność w 4 miastach, wersje językowe PL/EN/DE (klienci zagraniczni).</t>
+        </is>
+      </c>
+      <c r="N22" s="13" t="inlineStr">
+        <is>
+          <t>Adwokaci i doradcy podatkowi, nie radcowie prawni; wąski zakres (tylko sprawy karne skarbowe, nie cywilna odpowiedzialność z art. 299 KSH); brak opinii klientów; brak cen.</t>
+        </is>
+      </c>
+      <c r="O22" s="13" t="inlineStr">
+        <is>
+          <t>Wąska nisza (tylko karno-skarbowe) nie pokrywa całego zagrożenia klienta z pozwem cywilnym — KRS Guard może pozycjonować się jako kompleksowe rozwiązanie obejmujące też odpowiedzialność cywilną z art. 299 KSH.</t>
+        </is>
+      </c>
+      <c r="P22" s="13" t="inlineStr">
+        <is>
+          <t>Niskie dla głównego segmentu KRS Guard (inny typ sprawy — karna vs. cywilna), ale duży, wielojęzyczny zasięg może przechwytywać część klientów szukających szerzej "obrona zarządu".</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="150" customHeight="1"/>
+    <row r="24" ht="150" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
           <t>KRS Guard</t>
@@ -1663,6 +2565,46 @@
       <c r="H24" s="9" t="inlineStr">
         <is>
           <t>45 spraw — jedyna liczba na rynku dla tej konkretnej specjalizacji</t>
+        </is>
+      </c>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K24" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M24" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N24" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O24" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P24" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprostuj 4 bledne/wymyslone twierdzenia w arkuszu po weryfikacji na zywo w przegladarce (KSK, UpStart Legal, Jakubowska-Zawada, PW Restrukturyzacja) + dodaj ostrzezenie o rzetelnosci
</commit_message>
<xml_diff>
--- a/plany/lista-konkurencji-KRS-Guard-2026-08-05.xlsx
+++ b/plany/lista-konkurencji-KRS-Guard-2026-08-05.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,6 +72,12 @@
       <i val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -117,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -146,6 +152,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -513,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -676,6 +685,13 @@
       <c r="A21" t="inlineStr">
         <is>
           <t>Aktualizacja 05.08.2026: opisy Tier 1 zweryfikowane z pierwszej reki (odwiedzenie realnych stron WWW, nie tylko domysl) + dodane opinie klientow, status radcy prawnego i pelna analiza SWOT (mocne/slabe strony konkurenta, szanse/zagrozenia dla KRS Guard) dla kazdej z 21 firm Tier 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="140" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>WAZNA UWAGA O RZETELNOSCI (06.08.2026): przy sprawdzeniu 4 losowo zakwestionowanych twierdzen z kolumny "Ciekawe pomysly dla KRS Guard" (KSK, UpStart Legal, Jakubowska-Zawada, PW Restrukturyzacja) poprzez zywe przegladanie stron - 2 z 4 okazaly sie CZESCIOWO LUB CALKOWICIE NIEPRAWDZIWE (wymyslone FAQ u Jakubowskiej-Zawady; wymyslone liczby case study u PW Restrukturyzacja), a jedno bylo istotnie niescisle (UpStart Legal opisany jako dzialajacy 'wylacznie zdalnie', mimo posiadania biura). Poprawiono te 4 wpisy z dokladnym opisem zrodla bledu. NIE oznacza to, ze reszta zestawienia (pozostale 17 firm, pozostale kolumny) jest bledna - ale skoro na tej malej probce wykryto ok. 50% trafien z bledem, KAZDE twierdzenie z tego arkusza, ktore ma trafic do materialow marketingowych lub decyzji biznesowych, warto samodzielnie zweryfikowac na zrodlowej stronie przed uzyciem.</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1585,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Konsultacja 400-600 zł brutto; pierwszy kontakt WARUNKOWO bezpłatny</t>
+          <t>PONOWNIE ZWERYFIKOWANE 06.08.2026 z live browsingu: kwota 400-600 zl POTWIERDZONA - jest na stronie glownej w rozwijanym FAQ "Jaki jest koszt obslugi prawnej?": "Jednorazowa porada i usluga prawna zwykle kosztuje od ok. 400 zl do ok. 600 zl brutto za jedna konsultacje." UWAGA: to OGOLNA odpowiedz o kosztach uslug calej kancelarii, NIE cena dedykowana konkretnie tematowi ochrony zarzadu - takiej osobnej ceny na stronie brak.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -1646,7 +1662,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>(a) WYŁĄCZNIE ZDALNIE — jedyna taka firma z 21</t>
+          <t>SPROSTOWANIE 06.08.2026 (live browsing): poprzedni zapis "WYLACZNIE ZDALNIE - jedyna taka firma z 21" byl NIEScISLY. Na stronie /kontakt/ podany jest realny adres fizycznego biura: "ul. Mieleckiego 10 lok.305, 40-013 Katowice" (z linkiem "Zobacz na mapie"). To wiec (b) model hybrydowy - biuro stacjonarne + obsluga zdalna, NIE praca wylacznie zdalna bez biura.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -1681,12 +1697,12 @@
       </c>
       <c r="L12" s="13" t="inlineStr">
         <is>
-          <t>CZESCIOWO ZAWYZONE: cennik (150 zl konsultacja / 500 zl sprawdzenie wniosku / od 5500 zl pelna obsluga) potwierdzony aktualny, ALE dotyczy uslugi upadlosci konsumenckiej, nie osobno wycenionej ochrony zarzadu - laczenie mylace. "Niemal wylacznie ten temat" - przesadzone, to 1 z 6 rownorzednych uslug.</t>
+          <t>SPROSTOWANE 06.08.2026: pierwotny opis modelu obslugi ("wylacznie zdalnie") byl bledny - firma ma fizyczne biuro w Katowicach (patrz kolumna "Model obslugi"). Wszystkie pozostale ustalenia (radca prawny niejawny, cennik, "1 z 6 uslug") - bez zmian, potwierdzone wczesniej.</t>
         </is>
       </c>
       <c r="M12" s="13" t="inlineStr">
         <is>
-          <t>JEDYNA firma w Tier 1 działająca wyłącznie zdalnie (jak KRS Guard), jawny, rozpisany cennik (4 warianty), lead magnet "sprawdź swoją zdolność upadłościową".</t>
+          <t>Jawny, rozpisany cennik (4 warianty), lead magnet "sprawdz swoja zdolnosc upadlosciowa". UWAGA: wczesniej blednie wpisany "model wylacznie zdalny" jako mocna strona zostal usuniety po sprostowaniu - patrz kolumna "Model obslugi".</t>
         </is>
       </c>
       <c r="N12" s="13" t="inlineStr">
@@ -1701,7 +1717,7 @@
       </c>
       <c r="P12" s="13" t="inlineStr">
         <is>
-          <t>JEDYNY realny konkurent z tym samym modelem obsługi (wyłącznie zdalnie) i podobnym podejściem do jawności cen — warto obserwować, czy nie rozwinie mocniej właśnie tego tematu.</t>
+          <t>SPROSTOWANE: skoro UpStart Legal jednak MA fizyczne biuro (nie jest w pelni zdalna), oznacza to, ze WSROD 21 SPRAWDZONYCH FIRM ZADNA nie dziala w modelu identycznym z KRS Guard (wylacznie zdalnie, bez zadnego biura) - to jeszcze mocniejszy, bardziej unikalny wyroznik KRS Guard niz wczesniej sadzono, nie zagrozenie.</t>
         </is>
       </c>
     </row>
@@ -2004,7 +2020,7 @@
       </c>
       <c r="K16" s="13" t="inlineStr">
         <is>
-          <t>Krotkie "W skrocie" podsumowanie na gorze kazdej podstrony uslugowej (2-3 zdania przed pelnym tekstem) - dobry wzorzec UX. Rozbudowane FAQ tlumaczace roznice adwokat/radca prawny/kancelaria odszkodowawcza.</t>
+          <t>SPROSTOWANE 06.08.2026 (live browsing calej strony + menu nawigacji): "Rozbudowane FAQ tlumaczace roznice adwokat/radca prawny/kancelaria odszkodowawcza" - NIE ZNALEZIONE, wycofane. Sprawdzona strona /ochrona-czlonkow-zarzadu/ w calosci (pelne odczytanie struktury strony) oraz menu calej witryny (Obszary Doradztwa, Specjalizacje, Studium Przypadku, Publikacje, Kontakt) - nigdzie nie ma sekcji FAQ ani takiego porownania. To byl blad poprzedniej weryfikacji. POTWIERDZONE i pozostaje w mocy: krotkie podsumowanie "W skrocie:" na poczatku artykulu (cytat: "W skrocie: Ochrona prawna czlonka zarzadu obejmuje obrone przed odpowiedzialnoscia cywilna za zobowiazania spolki...") - to jest realny, dobry wzorzec UX wart rozwazenia.</t>
         </is>
       </c>
       <c r="L16" s="13" t="inlineStr">
@@ -2086,7 +2102,7 @@
       </c>
       <c r="K17" s="13" t="inlineStr">
         <is>
-          <t>Case studies z konkretnymi liczbami ("Suma korzysci dla klienta: 291 734 zl", "Czas realizacji: 83 dni") - bardzo przekonujacy format social proof, wart skopiowania. Artykul-"test" ("Kiedy ryzykujesz prywatnym majatkiem? [Test]") jako format angazujacy.</t>
+          <t>SPROSTOWANE 06.08.2026 (live browsing strony glownej, sekcji "Studium przypadku" w calosci): liczby "Suma korzysci dla klienta: 291 734 zl" i "Czas realizacji: 83 dni" - NIE ZNALEZIONE, wycofane. Na stronie jest tylko JEDNO studium przypadku - "Sprawnie przeprowadzona restrukturyzacja w malym gospodarstwie rolnym" - dotyczy INNEJ uslugi (restrukturyzacja firmy rolnej, nie ochrony czlonkow zarzadu) i zawiera WYLACZNIE opisowe, jakosciowe rezultaty ("poprawa plynnosci finansowej", "ochrona przed bankructwem"), BEZ zadnych liczb. To byl blad poprzedniej weryfikacji - zrodlo tych konkretnych liczb nie zostalo odnalezione na stronie. POTWIERDZONE i pozostaje w mocy: artykul-"test" pt. "Odpowiedzialnosc zarzadu za dlugi spolki: Kiedy ryzykujesz prywatnym majatkiem? [Test]" istnieje naprawde (link potwierdzony na podstronie uslugi ochrony zarzadu).</t>
         </is>
       </c>
       <c r="L17" s="13" t="inlineStr">
@@ -2096,7 +2112,7 @@
       </c>
       <c r="M17" s="13" t="inlineStr">
         <is>
-          <t>NAJLEPIEJ potwierdzony wpis w całym zestawieniu: dedykowana usługa w menu, realne imienne opinie 5-gwiazdkowe, case studies z konkretnymi liczbami (kwoty korzyści, czas realizacji), radcowie prawni na czele, jasno opisany proces w 6 krokach.</t>
+          <t>Dedykowana usluga w menu, realne imienne opinie 5-gwiazdkowe na stronie glownej, radcowie prawni na czele, jasno opisany proces w 6 krokach. SPROSTOWANE: wczesniejsza wzmianka o "case studies z konkretnymi liczbami" zostala usunieta - nie zostala potwierdzona na stronie (patrz kolumna "Ciekawe pomysly").</t>
         </is>
       </c>
       <c r="N17" s="13" t="inlineStr">
@@ -2111,7 +2127,7 @@
       </c>
       <c r="P17" s="13" t="inlineStr">
         <is>
-          <t>Razem ze Staniek&amp;Partners NAJSILNIEJSZY konkurent contentowo i wizerunkowo w całym zestawieniu — kompletna, w pełni potwierdzona oferta + dowód społeczny + liczbowe case studies.</t>
+          <t>Nadal solidny, kompletny konkurent (dedykowana usluga, radcowie prawni, realne opinie), ale SLABIEJ potwierdzony niz wczesniej sadzono - kluczowy argument "case studies z liczbami" okazal sie niepotwierdzony przy ponownej weryfikacji.</t>
         </is>
       </c>
     </row>

</xml_diff>